<commit_message>
update to SpineOpt v0.11.4
</commit_message>
<xml_diff>
--- a/SpineOptInputConfigs/System-MGA-invest-builder.xlsx
+++ b/SpineOptInputConfigs/System-MGA-invest-builder.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ethz-my.sharepoint.com/personal/jiahuang_ethz_ch/Documents/Desktop/ESA D-MAVT/PhD research/ModellingLocal/ESAurban-SpineOpt/SpineOptInputConfigs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="112" documentId="11_69E2A32EA847B44E2B09CAFD4C3FA92527743FA3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1983D009-6C43-4B1F-8695-7AAD3E9449D9}"/>
+  <xr:revisionPtr revIDLastSave="122" documentId="11_69E2A32EA847B44E2B09CAFD4C3FA92527743FA3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBA07A0F-4A11-46AD-AD1D-516E8D893785}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="5100" windowWidth="38640" windowHeight="21840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="unit" sheetId="1" r:id="rId1"/>

</xml_diff>